<commit_message>
New now safe point
</commit_message>
<xml_diff>
--- a/МРиПЭ/Киссофт/load.xlsx
+++ b/МРиПЭ/Киссофт/load.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="6" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="9" uniqueCount="3">
   <si>
     <t>Frequency_percent</t>
   </si>
@@ -88,7 +88,7 @@
     </row>
     <row r="2">
       <c r="A2" s="0">
-        <v>0.0075524735321598471</v>
+        <v>0.0022106007544945264</v>
       </c>
       <c r="B2" s="0">
         <v>0.24942003205142174</v>
@@ -99,7 +99,7 @@
     </row>
     <row r="3">
       <c r="A3" s="0">
-        <v>0.012909319958229136</v>
+        <v>0.0050966409853528717</v>
       </c>
       <c r="B3" s="0">
         <v>0.872970112179976</v>
@@ -110,7 +110,7 @@
     </row>
     <row r="4">
       <c r="A4" s="0">
-        <v>0.020735179437736361</v>
+        <v>0.010665129307574253</v>
       </c>
       <c r="B4" s="0">
         <v>1.4965201923085303</v>
@@ -121,7 +121,7 @@
     </row>
     <row r="5">
       <c r="A5" s="0">
-        <v>0.031297015256998101</v>
+        <v>0.020256244952794364</v>
       </c>
       <c r="B5" s="0">
         <v>1.9732020921817923</v>
@@ -132,7 +132,7 @@
     </row>
     <row r="6">
       <c r="A6" s="0">
-        <v>0.044390403622483102</v>
+        <v>0.034919223207262352</v>
       </c>
       <c r="B6" s="0">
         <v>1.9999999901918553</v>
@@ -143,7 +143,7 @@
     </row>
     <row r="7">
       <c r="A7" s="0">
-        <v>0.059165238578886399</v>
+        <v>0.054636744639326218</v>
       </c>
       <c r="B7" s="0">
         <v>1.9999999920193616</v>
@@ -154,7 +154,7 @@
     </row>
     <row r="8">
       <c r="A8" s="0">
-        <v>0.074102993441049647</v>
+        <v>0.077592750218062889</v>
       </c>
       <c r="B8" s="0">
         <v>1.9999999932716868</v>
@@ -165,7 +165,7 @@
     </row>
     <row r="9">
       <c r="A9" s="0">
-        <v>0.087216104923006854</v>
+        <v>0.10001720918815929</v>
       </c>
       <c r="B9" s="0">
         <v>1.9999999941837929</v>
@@ -176,7 +176,7 @@
     </row>
     <row r="10">
       <c r="A10" s="0">
-        <v>0.096460513400145304</v>
+        <v>0.11701631698570313</v>
       </c>
       <c r="B10" s="0">
         <v>1.9999999948778799</v>
@@ -187,7 +187,7 @@
     </row>
     <row r="11">
       <c r="A11" s="0">
-        <v>0.10025233265472069</v>
+        <v>0.12426154536550396</v>
       </c>
       <c r="B11" s="0">
         <v>1.9999999954238343</v>
@@ -198,7 +198,7 @@
     </row>
     <row r="12">
       <c r="A12" s="0">
-        <v>0.09791099712197146</v>
+        <v>0.11976941013214223</v>
       </c>
       <c r="B12" s="0">
         <v>1.9999999958645371</v>
@@ -209,7 +209,7 @@
     </row>
     <row r="13">
       <c r="A13" s="0">
-        <v>0.089858778153303967</v>
+        <v>0.10477888723679157</v>
       </c>
       <c r="B13" s="0">
         <v>1.9999999962277657</v>
@@ -220,7 +220,7 @@
     </row>
     <row r="14">
       <c r="A14" s="0">
-        <v>0.077496398085315901</v>
+        <v>0.083199346496101612</v>
       </c>
       <c r="B14" s="0">
         <v>1.999999996532309</v>
@@ -231,7 +231,7 @@
     </row>
     <row r="15">
       <c r="A15" s="0">
-        <v>0.062805021550719972</v>
+        <v>0.059963025564797788</v>
       </c>
       <c r="B15" s="0">
         <v>1.9999999967913325</v>
@@ -242,7 +242,7 @@
     </row>
     <row r="16">
       <c r="A16" s="0">
-        <v>0.047829834521130744</v>
+        <v>0.039225054782875815</v>
       </c>
       <c r="B16" s="0">
         <v>1.9999999970143345</v>
@@ -253,7 +253,7 @@
     </row>
     <row r="17">
       <c r="A17" s="0">
-        <v>0.034229046934842709</v>
+        <v>0.023289414518081853</v>
       </c>
       <c r="B17" s="0">
         <v>1.9999999972083446</v>
@@ -264,7 +264,7 @@
     </row>
     <row r="18">
       <c r="A18" s="0">
-        <v>0.023018756684593869</v>
+        <v>0.01255066849606948</v>
       </c>
       <c r="B18" s="0">
         <v>1.9999999973786722</v>
@@ -275,7 +275,7 @@
     </row>
     <row r="19">
       <c r="A19" s="0">
-        <v>0.01454653978204953</v>
+        <v>0.0061388412965802559</v>
       </c>
       <c r="B19" s="0">
         <v>1.9999999975294054</v>
@@ -286,7 +286,7 @@
     </row>
     <row r="20">
       <c r="A20" s="0">
-        <v>0.0086382927676792905</v>
+        <v>0.00272530369111071</v>
       </c>
       <c r="B20" s="0">
         <v>1.9999999976637421</v>
@@ -297,7 +297,7 @@
     </row>
     <row r="21">
       <c r="A21" s="0">
-        <v>0.0048204332404850328</v>
+        <v>0.0010981199029806367</v>
       </c>
       <c r="B21" s="0">
         <v>2.0226353752682811</v>
@@ -308,7 +308,7 @@
     </row>
     <row r="22">
       <c r="A22" s="0">
-        <v>0.0025277473226693035</v>
+        <v>0.00040159483596931961</v>
       </c>
       <c r="B22" s="0">
         <v>2.1208981015165214</v>
@@ -319,7 +319,7 @@
     </row>
     <row r="23">
       <c r="A23" s="0">
-        <v>0.0012455757023601558</v>
+        <v>0.00013329898815782221</v>
       </c>
       <c r="B23" s="0">
         <v>2.2248636947281155</v>
@@ -330,7 +330,7 @@
     </row>
     <row r="24">
       <c r="A24" s="0">
-        <v>0.00057675966249220827</v>
+        <v>4.0157123321336821e-05</v>
       </c>
       <c r="B24" s="0">
         <v>2.3288292879397097</v>
@@ -341,7 +341,7 @@
     </row>
     <row r="25">
       <c r="A25" s="0">
-        <v>0.00025096159450380378</v>
+        <v>1.0979732084583667e-05</v>
       </c>
       <c r="B25" s="0">
         <v>2.4327948811513043</v>
@@ -352,7 +352,7 @@
     </row>
     <row r="26">
       <c r="A26" s="0">
-        <v>0.00010261399386708497</v>
+        <v>2.7246484748648278e-06</v>
       </c>
       <c r="B26" s="0">
         <v>2.536760474362898</v>
@@ -363,7 +363,7 @@
     </row>
     <row r="27">
       <c r="A27" s="0">
-        <v>3.9426853344455901e-05</v>
+        <v>6.1364157763356464e-07</v>
       </c>
       <c r="B27" s="0">
         <v>2.6407260675744926</v>
@@ -374,7 +374,7 @@
     </row>
     <row r="28">
       <c r="A28" s="0">
-        <v>1.4235183145844292e-05</v>
+        <v>1.254297122818488e-07</v>
       </c>
       <c r="B28" s="0">
         <v>2.7446916607860863</v>
@@ -385,7 +385,7 @@
     </row>
     <row r="29">
       <c r="A29" s="0">
-        <v>4.8296825770003934e-06</v>
+        <v>2.3268213306679414e-08</v>
       </c>
       <c r="B29" s="0">
         <v>2.8486572539976804</v>
@@ -396,7 +396,7 @@
     </row>
     <row r="30">
       <c r="A30" s="0">
-        <v>1.5397770285748613e-06</v>
+        <v>3.9174013021294584e-09</v>
       </c>
       <c r="B30" s="0">
         <v>2.952622847209275</v>
@@ -407,7 +407,7 @@
     </row>
     <row r="31">
       <c r="A31" s="0">
-        <v>4.6129621703634859e-07</v>
+        <v>5.9855052811960107e-10</v>
       </c>
       <c r="B31" s="0">
         <v>3.0565884404208692</v>
@@ -418,7 +418,7 @@
     </row>
     <row r="32">
       <c r="A32" s="0">
-        <v>1.2986251538419989e-07</v>
+        <v>8.299778183163201e-11</v>
       </c>
       <c r="B32" s="0">
         <v>3.1605540336324629</v>
@@ -429,7 +429,7 @@
     </row>
     <row r="33">
       <c r="A33" s="0">
-        <v>3.4353311211457606e-08</v>
+        <v>1.0444559733597199e-11</v>
       </c>
       <c r="B33" s="0">
         <v>3.2645196268440571</v>
@@ -440,7 +440,7 @@
     </row>
     <row r="34">
       <c r="A34" s="0">
-        <v>8.5395158923793424e-09</v>
+        <v>1.192797584321057e-12</v>
       </c>
       <c r="B34" s="0">
         <v>3.3684852200556525</v>
@@ -451,7 +451,7 @@
     </row>
     <row r="35">
       <c r="A35" s="0">
-        <v>1.9946959126974723e-09</v>
+        <v>1.2362070563483479e-13</v>
       </c>
       <c r="B35" s="0">
         <v>3.4724508132672454</v>
@@ -462,7 +462,7 @@
     </row>
     <row r="36">
       <c r="A36" s="0">
-        <v>4.378222779600958e-10</v>
+        <v>1.1626750860800198e-14</v>
       </c>
       <c r="B36" s="0">
         <v>3.5764164064788395</v>
@@ -473,7 +473,7 @@
     </row>
     <row r="37">
       <c r="A37" s="0">
-        <v>9.6425929968116452e-11</v>
+        <v>1.0260798785027591e-15</v>
       </c>
       <c r="B37" s="0">
         <v>3.6907785590115929</v>

</xml_diff>